<commit_message>
feat(Q3): connect live NSE site to populate FY27_Q3 announced dates and mark unannounced as 'Yet to come'
</commit_message>
<xml_diff>
--- a/NSE_Official_Upcoming_Result_Dates.xlsx
+++ b/NSE_Official_Upcoming_Result_Dates.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarter Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nifty 50 Upcoming Result Dates'!$A$1:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All NSE Result Dates'!$A$1:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nifty 50 Upcoming Result Dates'!$A$1:$H$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All NSE Result Dates'!$A$1:$I$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -490,16 +490,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="31" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -551,17 +551,17 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>HCL Technologies Limited</t>
+          <t>Tata Consultancy Services Limited</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>12-Oct-2026 (Mon)</t>
+          <t>08-Oct-2026 (Thu)</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -571,7 +571,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>21d</t>
+          <t>14d</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -591,17 +591,17 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Axis Bank Limited</t>
+          <t>HCL Technologies Limited</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>17-Oct-2026 (Sat)</t>
+          <t>12-Oct-2026 (Mon)</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -611,12 +611,12 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>26d</t>
+          <t>18d</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Financial Results</t>
+          <t>Financial Results/Dividend</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -631,17 +631,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>UltraTech Cement Limited</t>
+          <t>HDFC Bank Limited</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>19-Oct-2026 (Mon)</t>
+          <t>17-Oct-2026 (Sat)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>28d</t>
+          <t>23d</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -671,42 +671,242 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>17-Oct-2026 (Sat)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>23d</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>17-Oct-2026 (Sat)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>23d</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>19-Oct-2026 (Mon)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>25d</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
           <t>INFY</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Infosys Limited</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>23-Oct-2026 (Fri)</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>32d</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>29d</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Financial Results/Dividend</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Dr. Reddy's Laboratories Limited</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>23-Oct-2026 (Fri)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>29d</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Mahindra &amp; Mahindra Limited</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>05-Nov-2026 (Thu)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>42d</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Financial Results/Other business matters</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>NSE Event Calendar API</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H5"/>
+  <autoFilter ref="A1:H10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -717,12 +917,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="31" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
@@ -784,17 +984,17 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>ANNU</t>
+          <t>MOMSBELIEF</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Annu Projects Limited</t>
+          <t>Rays of Belief Limited</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>23-Sep-2026 (Wed)</t>
+          <t>28-Sep-2026 (Mon)</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
@@ -804,7 +1004,7 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>2d</t>
+          <t>4d</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
@@ -829,17 +1029,17 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>WINSOME</t>
+          <t>PRASOLCHEM</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Winsome Yarns Limited</t>
+          <t>Prasol Chemicals Limited</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>23-Sep-2026 (Wed)</t>
+          <t>28-Sep-2026 (Mon)</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -849,7 +1049,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2d</t>
+          <t>4d</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -859,7 +1059,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Financial Results/Other business matters</t>
+          <t>Financial Results</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -869,45 +1069,45 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>HCLTECH</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>HCL Technologies Limited</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>12-Oct-2026 (Mon)</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>21d</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Financial Results/Dividend</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>DEEPA</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Deepa Jewellers Limited</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>28-Sep-2026 (Mon)</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Q1 FY2026-27 (Apr-Jun 2026)</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>4d</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>NSE Event Calendar API</t>
         </is>
@@ -919,27 +1119,27 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>STCINDIA</t>
+          <t>ANSALAPI</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>The State Trading Corporation of India Limited</t>
+          <t>Ansal Properties &amp; Infrastructure Limited</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>13-Oct-2026 (Tue)</t>
+          <t>29-Sep-2026 (Tue)</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+          <t>Q1 FY2026-27 (Apr-Jun 2026)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>22d</t>
+          <t>5d</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -949,7 +1149,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Financial Results/Other business matters</t>
+          <t>Financial Results/Dividend</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -959,45 +1159,45 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>AXISBANK</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Axis Bank Limited</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>17-Oct-2026 (Sat)</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>26d</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Financial Results</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>BFUTILITIE</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>BF Utilities Limited</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>30-Sep-2026 (Wed)</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Q1 FY2026-27 (Apr-Jun 2026)</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>6d</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Other business matters</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>NSE Event Calendar API</t>
         </is>
@@ -1009,17 +1209,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>INDIACEM</t>
+          <t>STEAMHOUSE</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>The India Cements Limited</t>
+          <t>Steamhouse India Limited</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>17-Oct-2026 (Sat)</t>
+          <t>05-Oct-2026 (Mon)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1029,7 +1229,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>26d</t>
+          <t>11d</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1049,180 +1249,180 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>ULTRACEMCO</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>UltraTech Cement Limited</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>19-Oct-2026 (Mon)</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>28d</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>GMBREW</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>GM Breweries Limited</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>08-Oct-2026 (Thu)</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>14d</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>08-Oct-2026 (Thu)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>14d</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Financial Results</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>NSE Event Calendar API</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>COFORGE</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Coforge Limited</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>23-Oct-2026 (Fri)</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>32d</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Financial Results</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Financial Results/Dividend</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>NSE Event Calendar API</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>INFY</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Infosys Limited</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>23-Oct-2026 (Fri)</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>32d</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>CRAMC</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Canara Robeco Asset Management Company Limited</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>09-Oct-2026 (Fri)</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>15d</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>HCL Technologies Limited</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>12-Oct-2026 (Mon)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>18d</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Financial Results/Dividend</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>NSE Event Calendar API</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>SHREECEM</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>SHREE CEMENT LIMITED</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>23-Oct-2026 (Fri)</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>32d</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Financial Results</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>NSE Event Calendar API</t>
         </is>
@@ -1234,47 +1434,1307 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
+          <t>ICICIPRULI</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>ICICI Prudential Life Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>13-Oct-2026 (Tue)</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>19d</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>STCINDIA</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>The State Trading Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>13-Oct-2026 (Tue)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>19d</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results/Other business matters</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>TATATECH</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Tata Technologies Limited</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>14-Oct-2026 (Wed)</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>20d</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>HDFCAMC</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>HDFC Asset Management Company Limited</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>15-Oct-2026 (Thu)</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>21d</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>ANGELONE</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Angel One Limited</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>15-Oct-2026 (Thu)</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>21d</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>KARURVYSYA</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Karur Vysya Bank Limited</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>15-Oct-2026 (Thu)</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>21d</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>17-Oct-2026 (Sat)</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>23d</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>17-Oct-2026 (Sat)</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>23d</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>17-Oct-2026 (Sat)</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>23d</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>INDIACEM</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>The India Cements Limited</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>17-Oct-2026 (Sat)</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>23d</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>LTTS</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>L&amp;T Technology Services Limited</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>19-Oct-2026 (Mon)</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>25d</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results/Dividend</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>19-Oct-2026 (Mon)</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>25d</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>CIEINDIA</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>CIE Automotive India Limited</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>22-Oct-2026 (Thu)</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>28d</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>TMCV</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Tata Motors Limited</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>23-Oct-2026 (Fri)</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>29d</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>SHREE CEMENT LIMITED</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>23-Oct-2026 (Fri)</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>29d</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>UTIAMC</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>UTI Asset Management Company Limited</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>23-Oct-2026 (Fri)</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>29d</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results/Other business matters</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>23-Oct-2026 (Fri)</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>29d</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Financial Results/Dividend</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Reddy's Laboratories Limited</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>23-Oct-2026 (Fri)</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>29d</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>COFORGE</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Coforge Limited</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>23-Oct-2026 (Fri)</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>29d</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>BBL</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Bharat Bijlee Limited</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>27-Oct-2026 (Tue)</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>33d</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>NAVINFLUOR</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Navin Fluorine International Limited</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>30-Oct-2026 (Fri)</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>36d</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results/Dividend</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>TVTODAY</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>TV Today Network Limited</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>02-Nov-2026 (Mon)</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>39d</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>ENDURANCE</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Endurance Technologies Limited</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>03-Nov-2026 (Tue)</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>40d</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>KANSAINER</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Kansai Nerolac Paints Limited</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>04-Nov-2026 (Wed)</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>41d</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>DABUR</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Dabur India Limited</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>04-Nov-2026 (Wed)</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>41d</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results/Dividend</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>MPHASIS</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>MphasiS Limited</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>05-Nov-2026 (Thu)</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>42d</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Mahindra &amp; Mahindra Limited</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>05-Nov-2026 (Thu)</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>42d</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Financial Results/Other business matters</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>TTKPRESTIG</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>TTK Prestige Limited</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>06-Nov-2026 (Fri)</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>43d</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>NSE Event Calendar API</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
           <t>ABB</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C40" s="8" t="inlineStr">
         <is>
           <t>ABB India Limited</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t>13-Nov-2026 (Fri)</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>53d</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>Financial Results</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Q2 FY2026-27 (Jul-Sep 2026)</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>50d</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>Financial Results</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
         <is>
           <t>NSE Event Calendar API</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I12"/>
+  <autoFilter ref="A1:I40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1326,11 +2786,11 @@
         <v>0</v>
       </c>
       <c r="C2" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>23 Sep -&gt; 23 Sep 2026</t>
+          <t>28 Sep -&gt; 30 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -1341,14 +2801,14 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>12 Oct -&gt; 13 Nov 2026</t>
+          <t>05 Oct -&gt; 13 Nov 2026</t>
         </is>
       </c>
     </row>

</xml_diff>